<commit_message>
research: freeze Gate 6 human evaluation results
</commit_message>
<xml_diff>
--- a/reports/final_v2/gate6/review/gate6_primary_blind_review.xlsx
+++ b/reports/final_v2/gate6/review/gate6_primary_blind_review.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary review" sheetId="1" r:id="Rc350ebe8e6cf474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary review" sheetId="1" r:id="R19c03d7709cc423a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4213,15 +4213,29 @@
         <x:v>Updated the version of `lucide-react` to `1.23.0` to ensure compatibility with the latest features and bug fixes.</x:v>
       </x:c>
       <x:c r="H17" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I17" s="20" t="str"/>
-      <x:c r="J17" s="20" t="str"/>
-      <x:c r="K17" s="20" t="str"/>
-      <x:c r="L17" s="20" t="str"/>
-      <x:c r="M17" s="20" t="str"/>
-      <x:c r="N17" s="20" t="str"/>
-      <x:c r="O17" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I17" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J17" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K17" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L17" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M17" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N17" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O17" s="20" t="str">
+        <x:v>Correct version bump, but the generic compatibility claim is unsupported and does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="8" t="str">
@@ -9785,15 +9799,29 @@
 - Updated `@apollo/subgraph` to version `2.14.4`.</x:v>
       </x:c>
       <x:c r="H35" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I35" s="20" t="str"/>
-      <x:c r="J35" s="20" t="str"/>
-      <x:c r="K35" s="20" t="str"/>
-      <x:c r="L35" s="20" t="str"/>
-      <x:c r="M35" s="20" t="str"/>
-      <x:c r="N35" s="20" t="str"/>
-      <x:c r="O35" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I35" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J35" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K35" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L35" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M35" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N35" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O35" s="20" t="str">
+        <x:v>Correct dependency bumps, but bare version bullets do not fit the selected sample README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="72" customHeight="1">
       <x:c r="A36" s="8" t="str">
@@ -10371,15 +10399,29 @@
 Different package managers may require different handling of installation scripts. To accommodate this, a new script `install:ci` is added to `MonorepoTsProject`. This script is conditionally set based on the package manager being used, ensuring compatibility and avoiding potential issues with certain package managers like Yarn Berry.</x:v>
       </x:c>
       <x:c r="H37" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I37" s="20" t="str"/>
-      <x:c r="J37" s="20" t="str"/>
-      <x:c r="K37" s="20" t="str"/>
-      <x:c r="L37" s="20" t="str"/>
-      <x:c r="M37" s="20" t="str"/>
-      <x:c r="N37" s="20" t="str"/>
-      <x:c r="O37" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I37" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J37" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K37" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L37" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M37" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N37" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O37" s="20" t="str">
+        <x:v>Misstates install:ci as new and omits the Yarn install override and Bun resolution change.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="72" customHeight="1">
       <x:c r="A38" s="8" t="str">
@@ -12308,15 +12350,29 @@
         <x:v>Updated the version of `shadcn` from 4.14.0 to 4.14.1.</x:v>
       </x:c>
       <x:c r="H45" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I45" s="20" t="str"/>
-      <x:c r="J45" s="20" t="str"/>
-      <x:c r="K45" s="20" t="str"/>
-      <x:c r="L45" s="20" t="str"/>
-      <x:c r="M45" s="20" t="str"/>
-      <x:c r="N45" s="20" t="str"/>
-      <x:c r="O45" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I45" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J45" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K45" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L45" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M45" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N45" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O45" s="20" t="str">
+        <x:v>Correct version bump, but a standalone dependency note does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="72" customHeight="1">
       <x:c r="A46" s="8" t="str">
@@ -12881,15 +12937,29 @@
         <x:v>Updated the version of `shadcn` from 4.8.2 to 4.8.3.</x:v>
       </x:c>
       <x:c r="H47" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I47" s="20" t="str"/>
-      <x:c r="J47" s="20" t="str"/>
-      <x:c r="K47" s="20" t="str"/>
-      <x:c r="L47" s="20" t="str"/>
-      <x:c r="M47" s="20" t="str"/>
-      <x:c r="N47" s="20" t="str"/>
-      <x:c r="O47" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I47" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J47" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K47" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L47" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M47" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N47" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O47" s="20" t="str">
+        <x:v>Correct version bump, but a standalone dependency note does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
       <x:c r="A48" s="8" t="str">
@@ -13443,15 +13513,29 @@
         <x:v>Updated the version of `i18next` to `26.4.0` to take advantage of recent improvements and bug fixes.</x:v>
       </x:c>
       <x:c r="H50" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I50" s="20" t="str"/>
-      <x:c r="J50" s="20" t="str"/>
-      <x:c r="K50" s="20" t="str"/>
-      <x:c r="L50" s="20" t="str"/>
-      <x:c r="M50" s="20" t="str"/>
-      <x:c r="N50" s="20" t="str"/>
-      <x:c r="O50" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I50" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J50" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K50" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L50" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M50" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N50" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O50" s="20" t="str">
+        <x:v>Correct version bump, but the claimed improvements and bug fixes are not supported by the diff.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="72" customHeight="1">
       <x:c r="A51" s="8" t="str">
@@ -15255,15 +15339,29 @@
         <x:v>Updated the version of `lucide-react` from `1.20.0` to `1.21.0`. This update ensures compatibility with the latest features and bug fixes provided by the library.</x:v>
       </x:c>
       <x:c r="H58" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I58" s="20" t="str"/>
-      <x:c r="J58" s="20" t="str"/>
-      <x:c r="K58" s="20" t="str"/>
-      <x:c r="L58" s="20" t="str"/>
-      <x:c r="M58" s="20" t="str"/>
-      <x:c r="N58" s="20" t="str"/>
-      <x:c r="O58" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I58" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J58" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K58" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L58" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M58" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N58" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O58" s="20" t="str">
+        <x:v>Correct version bump, but the compatibility and bug-fix claim is unsupported and does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="72" customHeight="1">
       <x:c r="A59" s="8" t="str">
@@ -15783,15 +15881,29 @@
 - **shadcn**: Bumped from version 4.14.1 to 4.15.0</x:v>
       </x:c>
       <x:c r="H60" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I60" s="20" t="str"/>
-      <x:c r="J60" s="20" t="str"/>
-      <x:c r="K60" s="20" t="str"/>
-      <x:c r="L60" s="20" t="str"/>
-      <x:c r="M60" s="20" t="str"/>
-      <x:c r="N60" s="20" t="str"/>
-      <x:c r="O60" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I60" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J60" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K60" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L60" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M60" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N60" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O60" s="20" t="str">
+        <x:v>Correct dependency bumps, but the changelog-style list does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="72" customHeight="1">
       <x:c r="A61" s="8" t="str">
@@ -15933,15 +16045,29 @@
 The goal of this framework is to enable bespoke tooling to be built without having to first traverse the CDK Tree and Metadata to build a graph.</x:v>
       </x:c>
       <x:c r="H61" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I61" s="20" t="str"/>
-      <x:c r="J61" s="20" t="str"/>
-      <x:c r="K61" s="20" t="str"/>
-      <x:c r="L61" s="20" t="str"/>
-      <x:c r="M61" s="20" t="str"/>
-      <x:c r="N61" s="20" t="str"/>
-      <x:c r="O61" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I61" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J61" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K61" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L61" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M61" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N61" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O61" s="20" t="str">
+        <x:v>The generated CDK Graph description is unrelated to the new build-environment Dockerfile.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="72" customHeight="1">
       <x:c r="A62" s="8" t="str">
@@ -16233,15 +16359,29 @@
         <x:v>Updated the version of the `shadcn` dependency from 4.17.0 to 4.18.0.</x:v>
       </x:c>
       <x:c r="H62" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I62" s="20" t="str"/>
-      <x:c r="J62" s="20" t="str"/>
-      <x:c r="K62" s="20" t="str"/>
-      <x:c r="L62" s="20" t="str"/>
-      <x:c r="M62" s="20" t="str"/>
-      <x:c r="N62" s="20" t="str"/>
-      <x:c r="O62" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I62" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J62" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K62" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L62" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M62" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N62" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O62" s="20" t="str">
+        <x:v>Correct version bump, but a standalone dependency note does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="72" customHeight="1">
       <x:c r="A63" s="8" t="str">
@@ -17720,15 +17860,29 @@
         <x:v>- Developers using NestJS will benefit from more robust handling of HTTP responses, especially when dealing with errors that might have falsy status codes.</x:v>
       </x:c>
       <x:c r="H66" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I66" s="20" t="str"/>
-      <x:c r="J66" s="20" t="str"/>
-      <x:c r="K66" s="20" t="str"/>
-      <x:c r="L66" s="20" t="str"/>
-      <x:c r="M66" s="20" t="str"/>
-      <x:c r="N66" s="20" t="str"/>
-      <x:c r="O66" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I66" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J66" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K66" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L66" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M66" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N66" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O66" s="20" t="str">
+        <x:v>Correct behavior summary, but it does not belong in CONTRIBUTING.md and omits adapter-specific details.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="72" customHeight="1">
       <x:c r="A67" s="8" t="str">
@@ -19967,15 +20121,29 @@
         <x:v>Updated the version of the `undici` dependency from 8.4.0 to 8.4.1.</x:v>
       </x:c>
       <x:c r="H75" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I75" s="20" t="str"/>
-      <x:c r="J75" s="20" t="str"/>
-      <x:c r="K75" s="20" t="str"/>
-      <x:c r="L75" s="20" t="str"/>
-      <x:c r="M75" s="20" t="str"/>
-      <x:c r="N75" s="20" t="str"/>
-      <x:c r="O75" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I75" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J75" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K75" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L75" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M75" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N75" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O75" s="20" t="str">
+        <x:v>Correct version bump, but a standalone dependency note does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="72" customHeight="1">
       <x:c r="A76" s="8" t="str">
@@ -24005,15 +24173,29 @@
         <x:v>Updated the version of `lucide-react` to `1.33.0`. This update ensures compatibility with the latest features and bug fixes provided by the library.</x:v>
       </x:c>
       <x:c r="H90" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I90" s="20" t="str"/>
-      <x:c r="J90" s="20" t="str"/>
-      <x:c r="K90" s="20" t="str"/>
-      <x:c r="L90" s="20" t="str"/>
-      <x:c r="M90" s="20" t="str"/>
-      <x:c r="N90" s="20" t="str"/>
-      <x:c r="O90" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I90" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J90" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K90" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L90" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M90" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N90" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O90" s="20" t="str">
+        <x:v>Correct version bump, but the compatibility and bug-fix claim is unsupported and does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="72" customHeight="1">
       <x:c r="A91" s="8" t="str">
@@ -26549,15 +26731,29 @@
         <x:v>Updated the version of `lucide-react` to `1.31.0` to ensure compatibility with the latest features and bug fixes.</x:v>
       </x:c>
       <x:c r="H100" s="20" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="I100" s="20" t="str"/>
-      <x:c r="J100" s="20" t="str"/>
-      <x:c r="K100" s="20" t="str"/>
-      <x:c r="L100" s="20" t="str"/>
-      <x:c r="M100" s="20" t="str"/>
-      <x:c r="N100" s="20" t="str"/>
-      <x:c r="O100" s="20" t="str"/>
+        <x:v>approved</x:v>
+      </x:c>
+      <x:c r="I100" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J100" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K100" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L100" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M100" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N100" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="O100" s="20" t="str">
+        <x:v>Correct version bump, but the generic compatibility claim is unsupported and does not fit the README.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="72" customHeight="1">
       <x:c r="A101" s="8" t="str">

</xml_diff>